<commit_message>
Minor GUI improvements and bug fixes
</commit_message>
<xml_diff>
--- a/gui/template/Student Base Template.xlsx
+++ b/gui/template/Student Base Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruele\PycharmProjects\RueLee\Boston Education\bosvoiceton-gui\gui\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruele\PycharmProjects\RueLee\Boston_Education\bosvoiceton-gui\gui\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{951FF907-0732-45F7-BC44-A69BE796F273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB76466-2FE2-46B4-B11F-7AF1677F2E2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -105,9 +105,6 @@
     <t>Balance/Credit from last invoice:</t>
   </si>
   <si>
-    <t>4211 Wilshire Blvd., Suite 136</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -130,6 +127,9 @@
       </rPr>
       <t>: Boston Education | (Venmo: @bostonedu; Zelle - 213-500-0101)</t>
     </r>
+  </si>
+  <si>
+    <t>4055 Wilshire Blvd., Suite #400</t>
   </si>
 </sst>
 </file>
@@ -1016,7 +1016,7 @@
     </row>
     <row r="4" spans="2:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>21</v>
@@ -1064,7 +1064,7 @@
     </row>
     <row r="11" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="32" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C11" s="33"/>
       <c r="D11" s="33"/>

</xml_diff>